<commit_message>
Ultimos ajustes, dato monto desde FBL3N,subi cuadro una celda para arriba
</commit_message>
<xml_diff>
--- a/Remittance.xlsx
+++ b/Remittance.xlsx
@@ -5,15 +5,15 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unilever.sharepoint.com/sites/ColombiaCreditManagement/Shared Documents/Cash App/KNIME/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose-Ricardo.Morales\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A189EDD8-64F5-468B-B526-71B04FC2076E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A595DBB8-3087-4F3F-A988-B56B11C0F695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A89A92A7-09EA-4A1C-AB67-799DE62D0028}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A9C53F7A-01A3-4A1A-93D4-763B7FC7824A}"/>
   </bookViews>
   <sheets>
-    <sheet name="REMADV202508120820_1182089" sheetId="2" r:id="rId1"/>
+    <sheet name="REMADV202508291655_1183343" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029" concurrentManualCount="12"/>
   <extLst>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="686" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="202">
   <si>
     <t>Informe de Pago</t>
   </si>
@@ -50,13 +50,13 @@
     <t>Beneficiario 2 : Unilever Andina S.A.</t>
   </si>
   <si>
-    <t>No. Aviso.: 00584423</t>
+    <t>No. Aviso.: 00590139</t>
   </si>
   <si>
     <t xml:space="preserve">Per. Facturación: </t>
   </si>
   <si>
-    <t>Fecha Aviso: 11-08-2025</t>
+    <t>Fecha Aviso: 29-08-2025</t>
   </si>
   <si>
     <t>Información de Pago</t>
@@ -86,10 +86,10 @@
     <t>Sucursal: Bogota</t>
   </si>
   <si>
-    <t>Nro. Cheque: 3702815749</t>
-  </si>
-  <si>
-    <t>Fecha Pago: 11-08-2025</t>
+    <t>Nro. Cheque: 3702736775</t>
+  </si>
+  <si>
+    <t>Fecha Pago: 29-08-2025</t>
   </si>
   <si>
     <t>Tasa Cambio: 0.000000</t>
@@ -101,7 +101,7 @@
     <t>Cód. Interno Proveedor: 0000100576</t>
   </si>
   <si>
-    <t>Orden de Pago: PK003702815749</t>
+    <t>Orden de Pago: PK003702736775</t>
   </si>
   <si>
     <t xml:space="preserve">Fecha Tasa Cambio: </t>
@@ -260,10 +260,49 @@
     <t>Factura Comercial</t>
   </si>
   <si>
-    <t>'5133509797</t>
-  </si>
-  <si>
-    <t>'PMP1243434001</t>
+    <t>'5133526811</t>
+  </si>
+  <si>
+    <t>'PMP1249244001</t>
+  </si>
+  <si>
+    <t>'7701008009608</t>
+  </si>
+  <si>
+    <t>'Bod 960 Cross-Docking</t>
+  </si>
+  <si>
+    <t>'4632109353</t>
+  </si>
+  <si>
+    <t>'0</t>
+  </si>
+  <si>
+    <t>'</t>
+  </si>
+  <si>
+    <t>''</t>
+  </si>
+  <si>
+    <t>EN</t>
+  </si>
+  <si>
+    <t>0.000</t>
+  </si>
+  <si>
+    <t>'5133559019</t>
+  </si>
+  <si>
+    <t>'PMP1249258001</t>
+  </si>
+  <si>
+    <t>'4632109351</t>
+  </si>
+  <si>
+    <t>'5132904345</t>
+  </si>
+  <si>
+    <t>'PMP1249400002</t>
   </si>
   <si>
     <t>'7701008009196</t>
@@ -272,367 +311,331 @@
     <t>'Bodega 919 Cross Droking Bogotá</t>
   </si>
   <si>
-    <t>'4631642214</t>
-  </si>
-  <si>
-    <t>'0</t>
-  </si>
-  <si>
-    <t>'</t>
-  </si>
-  <si>
-    <t>''</t>
-  </si>
-  <si>
-    <t>EN</t>
-  </si>
-  <si>
-    <t>0.000</t>
-  </si>
-  <si>
-    <t>'5133505762</t>
-  </si>
-  <si>
-    <t>'PMP1243435001</t>
-  </si>
-  <si>
-    <t>'4631642215</t>
-  </si>
-  <si>
-    <t>'5133425133</t>
-  </si>
-  <si>
-    <t>'PMP1243436001</t>
-  </si>
-  <si>
-    <t>'4631642213</t>
-  </si>
-  <si>
-    <t>'5133444164</t>
-  </si>
-  <si>
-    <t>'PMP1243437002</t>
-  </si>
-  <si>
-    <t>'4631642217</t>
-  </si>
-  <si>
-    <t>'5133465213</t>
-  </si>
-  <si>
-    <t>'PMP1243438002</t>
-  </si>
-  <si>
-    <t>'4631642219</t>
-  </si>
-  <si>
-    <t>'5133410379</t>
-  </si>
-  <si>
-    <t>'PMP1243439002</t>
-  </si>
-  <si>
-    <t>'5133413335</t>
-  </si>
-  <si>
-    <t>'PMP1243546001</t>
-  </si>
-  <si>
-    <t>'5133353624</t>
-  </si>
-  <si>
-    <t>'PMP1243587001</t>
-  </si>
-  <si>
-    <t>'7701008009608</t>
-  </si>
-  <si>
-    <t>'Bod 960 Cross-Docking</t>
-  </si>
-  <si>
-    <t>'4631755059</t>
-  </si>
-  <si>
-    <t>'5132399713</t>
-  </si>
-  <si>
-    <t>'PMP1243639002</t>
-  </si>
-  <si>
-    <t>'4631630357</t>
+    <t>'4632027137</t>
+  </si>
+  <si>
+    <t>'5133490119</t>
+  </si>
+  <si>
+    <t>'PMP1249405001</t>
+  </si>
+  <si>
+    <t>'4632100695</t>
+  </si>
+  <si>
+    <t>'5133108726</t>
+  </si>
+  <si>
+    <t>'PMP1249557001</t>
+  </si>
+  <si>
+    <t>'4632109349</t>
+  </si>
+  <si>
+    <t>'5133559878</t>
+  </si>
+  <si>
+    <t>'PMP1249558002</t>
+  </si>
+  <si>
+    <t>'4632109354</t>
+  </si>
+  <si>
+    <t>'5133510025</t>
+  </si>
+  <si>
+    <t>'PMP1249559002</t>
+  </si>
+  <si>
+    <t>'4632066563</t>
+  </si>
+  <si>
+    <t>'5133550902</t>
+  </si>
+  <si>
+    <t>'PMP1249560001</t>
+  </si>
+  <si>
+    <t>'4632027135</t>
+  </si>
+  <si>
+    <t>'5133474648</t>
+  </si>
+  <si>
+    <t>'PMP1249561001</t>
+  </si>
+  <si>
+    <t>'4632027134</t>
+  </si>
+  <si>
+    <t>'5133513191</t>
+  </si>
+  <si>
+    <t>'PMP1249562001</t>
+  </si>
+  <si>
+    <t>'4632100692</t>
+  </si>
+  <si>
+    <t>'5133423397</t>
+  </si>
+  <si>
+    <t>'PMP1249563002</t>
+  </si>
+  <si>
+    <t>'5133544136</t>
+  </si>
+  <si>
+    <t>'PMP1249564001</t>
+  </si>
+  <si>
+    <t>'5133567944</t>
+  </si>
+  <si>
+    <t>'PMP1249565002</t>
+  </si>
+  <si>
+    <t>'4632027138</t>
+  </si>
+  <si>
+    <t>'5133446644</t>
+  </si>
+  <si>
+    <t>'PMP1249566001</t>
+  </si>
+  <si>
+    <t>'4632100696</t>
+  </si>
+  <si>
+    <t>'5132667367</t>
+  </si>
+  <si>
+    <t>'PMP1249894001</t>
+  </si>
+  <si>
+    <t>'7701008009455</t>
+  </si>
+  <si>
+    <t>'Bod 945 CEDI Cartagena</t>
+  </si>
+  <si>
+    <t>'4631938987</t>
+  </si>
+  <si>
+    <t>'5133433219</t>
+  </si>
+  <si>
+    <t>'PMP1249897001</t>
+  </si>
+  <si>
+    <t>'7701008109001</t>
+  </si>
+  <si>
+    <t>'Bod 900 Cross Doking Costa</t>
+  </si>
+  <si>
+    <t>'4632003302</t>
+  </si>
+  <si>
+    <t>'5133015257</t>
+  </si>
+  <si>
+    <t>'PMP1249898001</t>
+  </si>
+  <si>
+    <t>'4631865203</t>
+  </si>
+  <si>
+    <t>'5133460746</t>
+  </si>
+  <si>
+    <t>'PMP1249901001</t>
+  </si>
+  <si>
+    <t>'4631938985</t>
+  </si>
+  <si>
+    <t>'5133508297</t>
+  </si>
+  <si>
+    <t>'PMP1249972001</t>
+  </si>
+  <si>
+    <t>'4632066562</t>
+  </si>
+  <si>
+    <t>'5132449468</t>
+  </si>
+  <si>
+    <t>'PMP1249973001</t>
+  </si>
+  <si>
+    <t>'4632003298</t>
+  </si>
+  <si>
+    <t>'5133492585</t>
+  </si>
+  <si>
+    <t>'PMP1249974001</t>
+  </si>
+  <si>
+    <t>'4632003299</t>
+  </si>
+  <si>
+    <t>'5132740196</t>
+  </si>
+  <si>
+    <t>'PMP1249975001</t>
+  </si>
+  <si>
+    <t>'5133537183</t>
+  </si>
+  <si>
+    <t>'PMP1249976001</t>
+  </si>
+  <si>
+    <t>'4632003303</t>
+  </si>
+  <si>
+    <t>'5133500457</t>
+  </si>
+  <si>
+    <t>'PMP1250219001</t>
+  </si>
+  <si>
+    <t>'4632092530</t>
+  </si>
+  <si>
+    <t>'5133446704</t>
+  </si>
+  <si>
+    <t>'PMP1250222001</t>
+  </si>
+  <si>
+    <t>'4631938984</t>
+  </si>
+  <si>
+    <t>'5133428310</t>
+  </si>
+  <si>
+    <t>'PMP1250223001</t>
+  </si>
+  <si>
+    <t>'4631938983</t>
+  </si>
+  <si>
+    <t>'5132789191</t>
+  </si>
+  <si>
+    <t>'PMP1250224001</t>
+  </si>
+  <si>
+    <t>'5133584850</t>
+  </si>
+  <si>
+    <t>'PMP1250225001</t>
+  </si>
+  <si>
+    <t>'4631938988</t>
   </si>
   <si>
     <t>Nota Crédito</t>
   </si>
   <si>
-    <t>'2103646940</t>
-  </si>
-  <si>
-    <t>'0085489002001</t>
-  </si>
-  <si>
-    <t>'2103646941</t>
-  </si>
-  <si>
-    <t>'0085489003001</t>
-  </si>
-  <si>
-    <t>'2103646942</t>
-  </si>
-  <si>
-    <t>'0085489004001</t>
-  </si>
-  <si>
-    <t>'2103646943</t>
-  </si>
-  <si>
-    <t>'0085489005001</t>
-  </si>
-  <si>
-    <t>'2103646944</t>
-  </si>
-  <si>
-    <t>'0085489006001</t>
-  </si>
-  <si>
-    <t>'2103646945</t>
-  </si>
-  <si>
-    <t>'0085489007001</t>
-  </si>
-  <si>
-    <t>'2103646946</t>
-  </si>
-  <si>
-    <t>'0085489008001</t>
-  </si>
-  <si>
-    <t>'2103646947</t>
-  </si>
-  <si>
-    <t>'0085489009001</t>
-  </si>
-  <si>
-    <t>'2103646948</t>
-  </si>
-  <si>
-    <t>'0085489010001</t>
-  </si>
-  <si>
-    <t>'2103646949</t>
-  </si>
-  <si>
-    <t>'0085489011001</t>
-  </si>
-  <si>
-    <t>'2103646950</t>
-  </si>
-  <si>
-    <t>'0085489012001</t>
-  </si>
-  <si>
-    <t>'2103646951</t>
-  </si>
-  <si>
-    <t>'0085489013001</t>
-  </si>
-  <si>
-    <t>'2103646952</t>
-  </si>
-  <si>
-    <t>'0085489014001</t>
-  </si>
-  <si>
-    <t>'2103646953</t>
-  </si>
-  <si>
-    <t>'0085489015001</t>
-  </si>
-  <si>
-    <t>'2103646954</t>
-  </si>
-  <si>
-    <t>'0085489016001</t>
-  </si>
-  <si>
-    <t>'2103646955</t>
-  </si>
-  <si>
-    <t>'0085489017001</t>
-  </si>
-  <si>
-    <t>'2103646956</t>
-  </si>
-  <si>
-    <t>'0085489018001</t>
-  </si>
-  <si>
-    <t>'2103637552</t>
-  </si>
-  <si>
-    <t>'0085489642001</t>
-  </si>
-  <si>
-    <t>'5213823879</t>
-  </si>
-  <si>
-    <t>'4631066394001</t>
-  </si>
-  <si>
-    <t>'7701008102026</t>
-  </si>
-  <si>
-    <t>Sto 202 Rodadero</t>
-  </si>
-  <si>
-    <t>'4631066394</t>
-  </si>
-  <si>
-    <t>'5213802054</t>
-  </si>
-  <si>
-    <t>'4633043274001</t>
-  </si>
-  <si>
-    <t>'7701008000575</t>
-  </si>
-  <si>
-    <t>STO 057 VILLA ADELA</t>
-  </si>
-  <si>
-    <t>'4633043274</t>
-  </si>
-  <si>
-    <t>'5213673573</t>
-  </si>
-  <si>
-    <t>'4633141222001</t>
-  </si>
-  <si>
-    <t>'7701008002272</t>
-  </si>
-  <si>
-    <t>STO 227 11 DE NOVIEMBRE</t>
-  </si>
-  <si>
-    <t>'4633141222</t>
-  </si>
-  <si>
-    <t>'5213755607</t>
-  </si>
-  <si>
-    <t>'4633373549001</t>
-  </si>
-  <si>
-    <t>'7701008009455</t>
+    <t>'5213419654</t>
+  </si>
+  <si>
+    <t>'4633807051001</t>
+  </si>
+  <si>
+    <t>'7701008003132</t>
+  </si>
+  <si>
+    <t>STO 313 CIENAGA DE ORO</t>
+  </si>
+  <si>
+    <t>'4633807051</t>
+  </si>
+  <si>
+    <t>'5213419655</t>
+  </si>
+  <si>
+    <t>'4634054712001</t>
+  </si>
+  <si>
+    <t>'7701008101128</t>
+  </si>
+  <si>
+    <t>Sao 112 San Felipe</t>
+  </si>
+  <si>
+    <t>'4634054712</t>
+  </si>
+  <si>
+    <t>'5313872796</t>
+  </si>
+  <si>
+    <t>'PMP1249400001</t>
+  </si>
+  <si>
+    <t>Bodega 919 Cross Droking Bogotá</t>
+  </si>
+  <si>
+    <t>'5314056670</t>
+  </si>
+  <si>
+    <t>'PMP1249558001</t>
+  </si>
+  <si>
+    <t>Bod 960 Cross-Docking</t>
+  </si>
+  <si>
+    <t>'5313592436</t>
+  </si>
+  <si>
+    <t>'PMP1249559001</t>
+  </si>
+  <si>
+    <t>'5314087548</t>
+  </si>
+  <si>
+    <t>'PMP1249563001</t>
+  </si>
+  <si>
+    <t>'5313928139</t>
+  </si>
+  <si>
+    <t>'PMP1249565001</t>
+  </si>
+  <si>
+    <t>'5314063653</t>
+  </si>
+  <si>
+    <t>'PMP1249972002</t>
+  </si>
+  <si>
+    <t>Bod 900 Cross Doking Costa</t>
+  </si>
+  <si>
+    <t>'5313978421</t>
+  </si>
+  <si>
+    <t>'PMP1249976002</t>
+  </si>
+  <si>
+    <t>'5314002274</t>
+  </si>
+  <si>
+    <t>'PMP1250219002</t>
   </si>
   <si>
     <t>Bod 945 CEDI Cartagena</t>
   </si>
   <si>
-    <t>'4633373549</t>
-  </si>
-  <si>
-    <t>'2103642620</t>
-  </si>
-  <si>
-    <t>'9801649295001</t>
-  </si>
-  <si>
-    <t>'2103664322</t>
-  </si>
-  <si>
-    <t>'9801649296001</t>
-  </si>
-  <si>
-    <t>'2103642621</t>
-  </si>
-  <si>
-    <t>'9801649297001</t>
-  </si>
-  <si>
-    <t>'2103642622</t>
-  </si>
-  <si>
-    <t>'9801649298001</t>
-  </si>
-  <si>
-    <t>'2103642623</t>
-  </si>
-  <si>
-    <t>'9801649299001</t>
-  </si>
-  <si>
-    <t>'2103766868</t>
-  </si>
-  <si>
-    <t>'9801649300001</t>
-  </si>
-  <si>
-    <t>'2103763867</t>
-  </si>
-  <si>
-    <t>'9801649301001</t>
-  </si>
-  <si>
-    <t>'2103623215</t>
-  </si>
-  <si>
-    <t>'9801649302001</t>
-  </si>
-  <si>
-    <t>'2103623216</t>
-  </si>
-  <si>
-    <t>'9801649303001</t>
-  </si>
-  <si>
-    <t>'2103623217</t>
-  </si>
-  <si>
-    <t>'9801649304001</t>
-  </si>
-  <si>
-    <t>'2103623218</t>
-  </si>
-  <si>
-    <t>'9801649305001</t>
-  </si>
-  <si>
-    <t>'5313971440</t>
-  </si>
-  <si>
-    <t>'PMP1243437001</t>
-  </si>
-  <si>
-    <t>Bodega 919 Cross Droking Bogotá</t>
-  </si>
-  <si>
-    <t>'5313918916</t>
-  </si>
-  <si>
-    <t>'PMP1243438001</t>
-  </si>
-  <si>
-    <t>'5314027710</t>
-  </si>
-  <si>
-    <t>'PMP1243439001</t>
-  </si>
-  <si>
-    <t>'5314044651</t>
-  </si>
-  <si>
-    <t>'PMP1243546002</t>
-  </si>
-  <si>
-    <t>'5313397965</t>
-  </si>
-  <si>
-    <t>'PMP1243639001</t>
-  </si>
-  <si>
-    <t>Bod 960 Cross-Docking</t>
+    <t>'5314088568</t>
+  </si>
+  <si>
+    <t>'PMP1250225002</t>
   </si>
   <si>
     <t>Totales.</t>
@@ -1532,8 +1535,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D57932B2-590F-4E8C-9DBA-C3FB4339EBB9}">
-  <dimension ref="A1:AN74"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93695156-669E-4955-A3B6-502E2BA8A89D}">
+  <dimension ref="A1:AN66"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35.5546875" bestFit="1" customWidth="1"/>
@@ -1555,7 +1558,7 @@
     <col min="17" max="17" width="10" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="9.77734375" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="8" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.33203125" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="7.33203125" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="7.5546875" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="7.6640625" bestFit="1" customWidth="1"/>
@@ -1748,12 +1751,14 @@
       <c r="B19" s="1" t="s">
         <v>33</v>
       </c>
+      <c r="N19" s="13"/>
     </row>
     <row r="20" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B20" s="3"/>
+      <c r="N20" s="13"/>
     </row>
     <row r="21" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A21" s="8"/>
@@ -1766,6 +1771,7 @@
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
+      <c r="N22" s="13"/>
     </row>
     <row r="23" spans="1:40" ht="12.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9"/>
@@ -1778,7 +1784,6 @@
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
-      <c r="N24" s="13"/>
     </row>
     <row r="25" spans="1:40" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="10"/>
@@ -1922,7 +1927,7 @@
         <v>76</v>
       </c>
       <c r="E27" s="12">
-        <v>45802</v>
+        <v>45819</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>77</v>
@@ -1949,16 +1954,16 @@
         <v>82</v>
       </c>
       <c r="N27" s="1">
-        <v>165989699</v>
+        <v>31277975</v>
       </c>
       <c r="O27" s="1">
-        <v>139487142</v>
+        <v>27002606</v>
       </c>
       <c r="P27" s="1">
         <v>0</v>
       </c>
       <c r="Q27" s="1">
-        <v>26502557</v>
+        <v>4275369</v>
       </c>
       <c r="R27" s="1">
         <v>0</v>
@@ -2022,7 +2027,7 @@
         <v>86</v>
       </c>
       <c r="E28" s="12">
-        <v>45802</v>
+        <v>45819</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>77</v>
@@ -2049,16 +2054,16 @@
         <v>82</v>
       </c>
       <c r="N28" s="1">
-        <v>29856410</v>
+        <v>1102345</v>
       </c>
       <c r="O28" s="1">
-        <v>25089420</v>
+        <v>926340</v>
       </c>
       <c r="P28" s="1">
         <v>0</v>
       </c>
       <c r="Q28" s="1">
-        <v>4766990</v>
+        <v>176005</v>
       </c>
       <c r="R28" s="1">
         <v>0</v>
@@ -2122,16 +2127,16 @@
         <v>89</v>
       </c>
       <c r="E29" s="12">
-        <v>45802</v>
+        <v>45819</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="I29" s="1" t="s">
         <v>80</v>
@@ -2149,16 +2154,16 @@
         <v>82</v>
       </c>
       <c r="N29" s="1">
-        <v>12528130</v>
+        <v>27692682</v>
       </c>
       <c r="O29" s="1">
-        <v>10527840</v>
+        <v>23902286</v>
       </c>
       <c r="P29" s="1">
         <v>0</v>
       </c>
       <c r="Q29" s="1">
-        <v>2000290</v>
+        <v>3790396</v>
       </c>
       <c r="R29" s="1">
         <v>0</v>
@@ -2216,22 +2221,22 @@
         <v>74</v>
       </c>
       <c r="C30" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E30" s="12">
+        <v>45819</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="G30" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D30" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="E30" s="12">
-        <v>45802</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>78</v>
-      </c>
       <c r="H30" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I30" s="1" t="s">
         <v>80</v>
@@ -2249,16 +2254,16 @@
         <v>82</v>
       </c>
       <c r="N30" s="1">
-        <v>83124</v>
+        <v>4992313</v>
       </c>
       <c r="O30" s="1">
-        <v>69852</v>
+        <v>4309915</v>
       </c>
       <c r="P30" s="1">
         <v>0</v>
       </c>
       <c r="Q30" s="1">
-        <v>13272</v>
+        <v>682398</v>
       </c>
       <c r="R30" s="1">
         <v>0</v>
@@ -2316,13 +2321,13 @@
         <v>74</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E31" s="12">
-        <v>45802</v>
+        <v>45819</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>77</v>
@@ -2331,7 +2336,7 @@
         <v>78</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="I31" s="1" t="s">
         <v>80</v>
@@ -2349,16 +2354,16 @@
         <v>82</v>
       </c>
       <c r="N31" s="1">
-        <v>53514044</v>
+        <v>20100423</v>
       </c>
       <c r="O31" s="1">
-        <v>44969785</v>
+        <v>16891112</v>
       </c>
       <c r="P31" s="1">
         <v>0</v>
       </c>
       <c r="Q31" s="1">
-        <v>8544259</v>
+        <v>3209311</v>
       </c>
       <c r="R31" s="1">
         <v>0</v>
@@ -2416,13 +2421,13 @@
         <v>74</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E32" s="12">
-        <v>45802</v>
+        <v>45819</v>
       </c>
       <c r="F32" s="1" t="s">
         <v>77</v>
@@ -2431,7 +2436,7 @@
         <v>78</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>79</v>
+        <v>101</v>
       </c>
       <c r="I32" s="1" t="s">
         <v>80</v>
@@ -2449,16 +2454,16 @@
         <v>82</v>
       </c>
       <c r="N32" s="1">
-        <v>757032037</v>
+        <v>72307698</v>
       </c>
       <c r="O32" s="1">
-        <v>636161375</v>
+        <v>60762772</v>
       </c>
       <c r="P32" s="1">
         <v>0</v>
       </c>
       <c r="Q32" s="1">
-        <v>120870662</v>
+        <v>11544926</v>
       </c>
       <c r="R32" s="1">
         <v>0</v>
@@ -2516,22 +2521,22 @@
         <v>74</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="E33" s="12">
-        <v>45803</v>
+        <v>45819</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="I33" s="1" t="s">
         <v>80</v>
@@ -2549,16 +2554,16 @@
         <v>82</v>
       </c>
       <c r="N33" s="1">
-        <v>122759901</v>
+        <v>94379986</v>
       </c>
       <c r="O33" s="1">
-        <v>103159581</v>
+        <v>79310913</v>
       </c>
       <c r="P33" s="1">
         <v>0</v>
       </c>
       <c r="Q33" s="1">
-        <v>19600320</v>
+        <v>15069073</v>
       </c>
       <c r="R33" s="1">
         <v>0</v>
@@ -2616,22 +2621,22 @@
         <v>74</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E34" s="12">
-        <v>45803</v>
+        <v>45819</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="I34" s="1" t="s">
         <v>80</v>
@@ -2649,16 +2654,16 @@
         <v>82</v>
       </c>
       <c r="N34" s="1">
-        <v>132622525</v>
+        <v>2263380</v>
       </c>
       <c r="O34" s="1">
-        <v>111447500</v>
+        <v>1902000</v>
       </c>
       <c r="P34" s="1">
         <v>0</v>
       </c>
       <c r="Q34" s="1">
-        <v>21175025</v>
+        <v>361380</v>
       </c>
       <c r="R34" s="1">
         <v>0</v>
@@ -2716,22 +2721,22 @@
         <v>74</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E35" s="12">
-        <v>45803</v>
+        <v>45819</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I35" s="1" t="s">
         <v>80</v>
@@ -2749,16 +2754,16 @@
         <v>82</v>
       </c>
       <c r="N35" s="1">
-        <v>343873745</v>
+        <v>79954317</v>
       </c>
       <c r="O35" s="1">
-        <v>288969533</v>
+        <v>67188501</v>
       </c>
       <c r="P35" s="1">
         <v>0</v>
       </c>
       <c r="Q35" s="1">
-        <v>54904212</v>
+        <v>12765816</v>
       </c>
       <c r="R35" s="1">
         <v>0</v>
@@ -2810,28 +2815,28 @@
     </row>
     <row r="36" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E36" s="12">
-        <v>45873</v>
+        <v>45819</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>81</v>
+        <v>113</v>
       </c>
       <c r="I36" s="1" t="s">
         <v>80</v>
@@ -2846,19 +2851,19 @@
         <v>81</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N36" s="1">
-        <v>-106616</v>
+        <v>19480076</v>
       </c>
       <c r="O36" s="1">
-        <v>-106616</v>
+        <v>16369812</v>
       </c>
       <c r="P36" s="1">
         <v>0</v>
       </c>
       <c r="Q36" s="1">
-        <v>0</v>
+        <v>3110264</v>
       </c>
       <c r="R36" s="1">
         <v>0</v>
@@ -2910,28 +2915,28 @@
     </row>
     <row r="37" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E37" s="12">
-        <v>45873</v>
+        <v>45819</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>81</v>
+        <v>110</v>
       </c>
       <c r="I37" s="1" t="s">
         <v>80</v>
@@ -2946,19 +2951,19 @@
         <v>81</v>
       </c>
       <c r="M37" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N37" s="1">
-        <v>-280732</v>
+        <v>122200697</v>
       </c>
       <c r="O37" s="1">
-        <v>-280732</v>
+        <v>102689662</v>
       </c>
       <c r="P37" s="1">
         <v>0</v>
       </c>
       <c r="Q37" s="1">
-        <v>0</v>
+        <v>19511035</v>
       </c>
       <c r="R37" s="1">
         <v>0</v>
@@ -3010,28 +3015,28 @@
     </row>
     <row r="38" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E38" s="12">
-        <v>45873</v>
+        <v>45819</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>81</v>
+        <v>113</v>
       </c>
       <c r="I38" s="1" t="s">
         <v>80</v>
@@ -3046,19 +3051,19 @@
         <v>81</v>
       </c>
       <c r="M38" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N38" s="1">
-        <v>-852931</v>
+        <v>7344450</v>
       </c>
       <c r="O38" s="1">
-        <v>-852931</v>
+        <v>6171807</v>
       </c>
       <c r="P38" s="1">
         <v>0</v>
       </c>
       <c r="Q38" s="1">
-        <v>0</v>
+        <v>1172643</v>
       </c>
       <c r="R38" s="1">
         <v>0</v>
@@ -3110,28 +3115,28 @@
     </row>
     <row r="39" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E39" s="12">
-        <v>45873</v>
+        <v>45819</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>81</v>
+        <v>120</v>
       </c>
       <c r="I39" s="1" t="s">
         <v>80</v>
@@ -3146,19 +3151,19 @@
         <v>81</v>
       </c>
       <c r="M39" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N39" s="1">
-        <v>-1235221</v>
+        <v>75077367</v>
       </c>
       <c r="O39" s="1">
-        <v>-1235221</v>
+        <v>63090225</v>
       </c>
       <c r="P39" s="1">
         <v>0</v>
       </c>
       <c r="Q39" s="1">
-        <v>0</v>
+        <v>11987142</v>
       </c>
       <c r="R39" s="1">
         <v>0</v>
@@ -3210,28 +3215,28 @@
     </row>
     <row r="40" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E40" s="12">
-        <v>45873</v>
+        <v>45819</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>81</v>
+        <v>123</v>
       </c>
       <c r="I40" s="1" t="s">
         <v>80</v>
@@ -3246,19 +3251,19 @@
         <v>81</v>
       </c>
       <c r="M40" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N40" s="1">
-        <v>-2772024</v>
+        <v>15478421</v>
       </c>
       <c r="O40" s="1">
-        <v>-2772024</v>
+        <v>13007077</v>
       </c>
       <c r="P40" s="1">
         <v>0</v>
       </c>
       <c r="Q40" s="1">
-        <v>0</v>
+        <v>2471344</v>
       </c>
       <c r="R40" s="1">
         <v>0</v>
@@ -3310,28 +3315,28 @@
     </row>
     <row r="41" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="E41" s="12">
-        <v>45873</v>
+        <v>45820</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>81</v>
+        <v>126</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>81</v>
+        <v>127</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>81</v>
+        <v>128</v>
       </c>
       <c r="I41" s="1" t="s">
         <v>80</v>
@@ -3346,19 +3351,19 @@
         <v>81</v>
       </c>
       <c r="M41" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N41" s="1">
-        <v>-3198490</v>
+        <v>5509234</v>
       </c>
       <c r="O41" s="1">
-        <v>-3198490</v>
+        <v>4756176</v>
       </c>
       <c r="P41" s="1">
         <v>0</v>
       </c>
       <c r="Q41" s="1">
-        <v>0</v>
+        <v>753058</v>
       </c>
       <c r="R41" s="1">
         <v>0</v>
@@ -3410,28 +3415,28 @@
     </row>
     <row r="42" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="E42" s="12">
-        <v>45873</v>
+        <v>45820</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>81</v>
+        <v>131</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>81</v>
+        <v>132</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>81</v>
+        <v>133</v>
       </c>
       <c r="I42" s="1" t="s">
         <v>80</v>
@@ -3446,19 +3451,19 @@
         <v>81</v>
       </c>
       <c r="M42" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N42" s="1">
-        <v>-4472640</v>
+        <v>11607265</v>
       </c>
       <c r="O42" s="1">
-        <v>-4472640</v>
+        <v>10020669</v>
       </c>
       <c r="P42" s="1">
         <v>0</v>
       </c>
       <c r="Q42" s="1">
-        <v>0</v>
+        <v>1586596</v>
       </c>
       <c r="R42" s="1">
         <v>0</v>
@@ -3510,28 +3515,28 @@
     </row>
     <row r="43" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="E43" s="12">
-        <v>45873</v>
+        <v>45820</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>81</v>
+        <v>126</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>81</v>
+        <v>127</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>81</v>
+        <v>136</v>
       </c>
       <c r="I43" s="1" t="s">
         <v>80</v>
@@ -3546,19 +3551,19 @@
         <v>81</v>
       </c>
       <c r="M43" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N43" s="1">
-        <v>-4895525</v>
+        <v>3747972</v>
       </c>
       <c r="O43" s="1">
-        <v>-4895525</v>
+        <v>3149557</v>
       </c>
       <c r="P43" s="1">
         <v>0</v>
       </c>
       <c r="Q43" s="1">
-        <v>0</v>
+        <v>598415</v>
       </c>
       <c r="R43" s="1">
         <v>0</v>
@@ -3610,28 +3615,28 @@
     </row>
     <row r="44" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A44" s="1">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="C44" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E44" s="12">
+        <v>45820</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="D44" s="1" t="s">
+      <c r="G44" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="E44" s="12">
-        <v>45873</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="G44" s="1" t="s">
-        <v>81</v>
-      </c>
       <c r="H44" s="1" t="s">
-        <v>81</v>
+        <v>139</v>
       </c>
       <c r="I44" s="1" t="s">
         <v>80</v>
@@ -3646,19 +3651,19 @@
         <v>81</v>
       </c>
       <c r="M44" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N44" s="1">
-        <v>-6266272</v>
+        <v>1322814</v>
       </c>
       <c r="O44" s="1">
-        <v>-6266272</v>
+        <v>1111608</v>
       </c>
       <c r="P44" s="1">
         <v>0</v>
       </c>
       <c r="Q44" s="1">
-        <v>0</v>
+        <v>211206</v>
       </c>
       <c r="R44" s="1">
         <v>0</v>
@@ -3710,28 +3715,28 @@
     </row>
     <row r="45" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="E45" s="12">
-        <v>45873</v>
+        <v>45820</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>81</v>
+        <v>131</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>81</v>
+        <v>132</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>81</v>
+        <v>142</v>
       </c>
       <c r="I45" s="1" t="s">
         <v>80</v>
@@ -3746,19 +3751,19 @@
         <v>81</v>
       </c>
       <c r="M45" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N45" s="1">
-        <v>-7156225</v>
+        <v>125839982</v>
       </c>
       <c r="O45" s="1">
-        <v>-7156225</v>
+        <v>105747884</v>
       </c>
       <c r="P45" s="1">
         <v>0</v>
       </c>
       <c r="Q45" s="1">
-        <v>0</v>
+        <v>20092098</v>
       </c>
       <c r="R45" s="1">
         <v>0</v>
@@ -3810,28 +3815,28 @@
     </row>
     <row r="46" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A46" s="1">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="D46" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E46" s="12">
+        <v>45820</v>
+      </c>
+      <c r="F46" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="E46" s="12">
-        <v>45873</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>81</v>
-      </c>
       <c r="G46" s="1" t="s">
-        <v>81</v>
+        <v>132</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>81</v>
+        <v>145</v>
       </c>
       <c r="I46" s="1" t="s">
         <v>80</v>
@@ -3846,19 +3851,19 @@
         <v>81</v>
       </c>
       <c r="M46" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N46" s="1">
-        <v>-7343319</v>
+        <v>28730082</v>
       </c>
       <c r="O46" s="1">
-        <v>-7343319</v>
+        <v>24142926</v>
       </c>
       <c r="P46" s="1">
         <v>0</v>
       </c>
       <c r="Q46" s="1">
-        <v>0</v>
+        <v>4587156</v>
       </c>
       <c r="R46" s="1">
         <v>0</v>
@@ -3910,28 +3915,28 @@
     </row>
     <row r="47" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A47" s="1">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="C47" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="E47" s="12">
+        <v>45820</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="G47" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D47" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="E47" s="12">
-        <v>45873</v>
-      </c>
-      <c r="F47" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="G47" s="1" t="s">
-        <v>81</v>
-      </c>
       <c r="H47" s="1" t="s">
-        <v>81</v>
+        <v>148</v>
       </c>
       <c r="I47" s="1" t="s">
         <v>80</v>
@@ -3946,19 +3951,19 @@
         <v>81</v>
       </c>
       <c r="M47" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N47" s="1">
-        <v>-16267041</v>
+        <v>3055563</v>
       </c>
       <c r="O47" s="1">
-        <v>-16267041</v>
+        <v>2567700</v>
       </c>
       <c r="P47" s="1">
         <v>0</v>
       </c>
       <c r="Q47" s="1">
-        <v>0</v>
+        <v>487863</v>
       </c>
       <c r="R47" s="1">
         <v>0</v>
@@ -4010,28 +4015,28 @@
     </row>
     <row r="48" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A48" s="1">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>135</v>
+        <v>150</v>
       </c>
       <c r="E48" s="12">
-        <v>45873</v>
+        <v>45820</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>81</v>
+        <v>131</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>81</v>
+        <v>132</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>81</v>
+        <v>145</v>
       </c>
       <c r="I48" s="1" t="s">
         <v>80</v>
@@ -4046,19 +4051,19 @@
         <v>81</v>
       </c>
       <c r="M48" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N48" s="1">
-        <v>-19679618</v>
+        <v>198843616</v>
       </c>
       <c r="O48" s="1">
-        <v>-19679618</v>
+        <v>167095476</v>
       </c>
       <c r="P48" s="1">
         <v>0</v>
       </c>
       <c r="Q48" s="1">
-        <v>0</v>
+        <v>31748140</v>
       </c>
       <c r="R48" s="1">
         <v>0</v>
@@ -4110,28 +4115,28 @@
     </row>
     <row r="49" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A49" s="1">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>136</v>
+        <v>151</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="E49" s="12">
-        <v>45873</v>
+        <v>45820</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>81</v>
+        <v>131</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>81</v>
+        <v>132</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>81</v>
+        <v>153</v>
       </c>
       <c r="I49" s="1" t="s">
         <v>80</v>
@@ -4146,19 +4151,19 @@
         <v>81</v>
       </c>
       <c r="M49" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N49" s="1">
-        <v>-22519415</v>
+        <v>86264216</v>
       </c>
       <c r="O49" s="1">
-        <v>-22519415</v>
+        <v>72490938</v>
       </c>
       <c r="P49" s="1">
         <v>0</v>
       </c>
       <c r="Q49" s="1">
-        <v>0</v>
+        <v>13773278</v>
       </c>
       <c r="R49" s="1">
         <v>0</v>
@@ -4210,28 +4215,28 @@
     </row>
     <row r="50" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A50" s="1">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>138</v>
+        <v>154</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
       <c r="E50" s="12">
-        <v>45873</v>
+        <v>45821</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>81</v>
+        <v>126</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>81</v>
+        <v>127</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>81</v>
+        <v>156</v>
       </c>
       <c r="I50" s="1" t="s">
         <v>80</v>
@@ -4246,19 +4251,19 @@
         <v>81</v>
       </c>
       <c r="M50" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N50" s="1">
-        <v>-24608350</v>
+        <v>62919991</v>
       </c>
       <c r="O50" s="1">
-        <v>-24608350</v>
+        <v>52873942</v>
       </c>
       <c r="P50" s="1">
         <v>0</v>
       </c>
       <c r="Q50" s="1">
-        <v>0</v>
+        <v>10046049</v>
       </c>
       <c r="R50" s="1">
         <v>0</v>
@@ -4310,28 +4315,28 @@
     </row>
     <row r="51" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A51" s="1">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>141</v>
+        <v>158</v>
       </c>
       <c r="E51" s="12">
-        <v>45873</v>
+        <v>45821</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>81</v>
+        <v>126</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>81</v>
+        <v>127</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>81</v>
+        <v>159</v>
       </c>
       <c r="I51" s="1" t="s">
         <v>80</v>
@@ -4346,19 +4351,19 @@
         <v>81</v>
       </c>
       <c r="M51" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N51" s="1">
-        <v>-63642284</v>
+        <v>2602887</v>
       </c>
       <c r="O51" s="1">
-        <v>-63642284</v>
+        <v>2187300</v>
       </c>
       <c r="P51" s="1">
         <v>0</v>
       </c>
       <c r="Q51" s="1">
-        <v>0</v>
+        <v>415587</v>
       </c>
       <c r="R51" s="1">
         <v>0</v>
@@ -4410,28 +4415,28 @@
     </row>
     <row r="52" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A52" s="1">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>142</v>
+        <v>160</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>143</v>
+        <v>161</v>
       </c>
       <c r="E52" s="12">
-        <v>45873</v>
+        <v>45821</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>81</v>
+        <v>126</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>81</v>
+        <v>127</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>81</v>
+        <v>162</v>
       </c>
       <c r="I52" s="1" t="s">
         <v>80</v>
@@ -4446,19 +4451,19 @@
         <v>81</v>
       </c>
       <c r="M52" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N52" s="1">
-        <v>-77643586</v>
+        <v>39567495</v>
       </c>
       <c r="O52" s="1">
-        <v>-77643586</v>
+        <v>33249996</v>
       </c>
       <c r="P52" s="1">
         <v>0</v>
       </c>
       <c r="Q52" s="1">
-        <v>0</v>
+        <v>6317499</v>
       </c>
       <c r="R52" s="1">
         <v>0</v>
@@ -4510,28 +4515,28 @@
     </row>
     <row r="53" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A53" s="1">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>144</v>
+        <v>163</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>145</v>
+        <v>164</v>
       </c>
       <c r="E53" s="12">
-        <v>45875</v>
+        <v>45821</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>81</v>
+        <v>126</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>81</v>
+        <v>127</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>81</v>
+        <v>162</v>
       </c>
       <c r="I53" s="1" t="s">
         <v>80</v>
@@ -4546,19 +4551,19 @@
         <v>81</v>
       </c>
       <c r="M53" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N53" s="1">
-        <v>-38727613</v>
+        <v>10928542</v>
       </c>
       <c r="O53" s="1">
-        <v>-38727613</v>
+        <v>9183648</v>
       </c>
       <c r="P53" s="1">
         <v>0</v>
       </c>
       <c r="Q53" s="1">
-        <v>0</v>
+        <v>1744894</v>
       </c>
       <c r="R53" s="1">
         <v>0</v>
@@ -4610,28 +4615,28 @@
     </row>
     <row r="54" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A54" s="1">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>146</v>
+        <v>165</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>147</v>
+        <v>166</v>
       </c>
       <c r="E54" s="12">
-        <v>45871</v>
+        <v>45821</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>148</v>
+        <v>126</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>149</v>
+        <v>127</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>150</v>
+        <v>167</v>
       </c>
       <c r="I54" s="1" t="s">
         <v>80</v>
@@ -4646,19 +4651,19 @@
         <v>81</v>
       </c>
       <c r="M54" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N54" s="1">
-        <v>-35833</v>
+        <v>34995137</v>
       </c>
       <c r="O54" s="1">
-        <v>-30112</v>
+        <v>29407678</v>
       </c>
       <c r="P54" s="1">
         <v>0</v>
       </c>
       <c r="Q54" s="1">
-        <v>-5721</v>
+        <v>5587459</v>
       </c>
       <c r="R54" s="1">
         <v>0</v>
@@ -4713,25 +4718,25 @@
         <v>381</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>109</v>
+        <v>168</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>151</v>
+        <v>169</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>152</v>
+        <v>170</v>
       </c>
       <c r="E55" s="12">
-        <v>45869</v>
+        <v>45897</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>153</v>
+        <v>171</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>154</v>
+        <v>172</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>155</v>
+        <v>173</v>
       </c>
       <c r="I55" s="1" t="s">
         <v>80</v>
@@ -4749,16 +4754,16 @@
         <v>81</v>
       </c>
       <c r="N55" s="1">
-        <v>-107500</v>
+        <v>-7083</v>
       </c>
       <c r="O55" s="1">
-        <v>-90336</v>
+        <v>-5952</v>
       </c>
       <c r="P55" s="1">
         <v>0</v>
       </c>
       <c r="Q55" s="1">
-        <v>-17164</v>
+        <v>-1131</v>
       </c>
       <c r="R55" s="1">
         <v>0</v>
@@ -4813,25 +4818,25 @@
         <v>381</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>109</v>
+        <v>168</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>157</v>
+        <v>175</v>
       </c>
       <c r="E56" s="12">
-        <v>45870</v>
+        <v>45897</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>158</v>
+        <v>176</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>159</v>
+        <v>177</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
       <c r="I56" s="1" t="s">
         <v>80</v>
@@ -4849,16 +4854,16 @@
         <v>81</v>
       </c>
       <c r="N56" s="1">
-        <v>-31860</v>
+        <v>-221909</v>
       </c>
       <c r="O56" s="1">
-        <v>-26773</v>
+        <v>-186478</v>
       </c>
       <c r="P56" s="1">
         <v>0</v>
       </c>
       <c r="Q56" s="1">
-        <v>-5087</v>
+        <v>-35431</v>
       </c>
       <c r="R56" s="1">
         <v>0</v>
@@ -4913,25 +4918,25 @@
         <v>381</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>109</v>
+        <v>168</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>161</v>
+        <v>179</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>162</v>
+        <v>180</v>
       </c>
       <c r="E57" s="12">
-        <v>45868</v>
+        <v>45819</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>163</v>
+        <v>90</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>164</v>
+        <v>181</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>165</v>
+        <v>92</v>
       </c>
       <c r="I57" s="1" t="s">
         <v>80</v>
@@ -4949,16 +4954,16 @@
         <v>81</v>
       </c>
       <c r="N57" s="1">
-        <v>-29575</v>
+        <v>-220481</v>
       </c>
       <c r="O57" s="1">
-        <v>-24853</v>
+        <v>-185278</v>
       </c>
       <c r="P57" s="1">
         <v>0</v>
       </c>
       <c r="Q57" s="1">
-        <v>-4722</v>
+        <v>-35203</v>
       </c>
       <c r="R57" s="1">
         <v>0</v>
@@ -5013,25 +5018,25 @@
         <v>381</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>109</v>
+        <v>168</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="E58" s="12">
-        <v>45873</v>
+        <v>45819</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>81</v>
+        <v>184</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>81</v>
+        <v>101</v>
       </c>
       <c r="I58" s="1" t="s">
         <v>80</v>
@@ -5049,16 +5054,16 @@
         <v>81</v>
       </c>
       <c r="N58" s="1">
-        <v>-817632</v>
+        <v>-96148</v>
       </c>
       <c r="O58" s="1">
-        <v>-701830</v>
+        <v>-80797</v>
       </c>
       <c r="P58" s="1">
         <v>0</v>
       </c>
       <c r="Q58" s="1">
-        <v>-133348</v>
+        <v>-15351</v>
       </c>
       <c r="R58" s="1">
         <v>0</v>
@@ -5067,7 +5072,7 @@
         <v>0</v>
       </c>
       <c r="T58" s="1">
-        <v>17546</v>
+        <v>0</v>
       </c>
       <c r="U58" s="1">
         <v>0</v>
@@ -5113,25 +5118,25 @@
         <v>381</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>109</v>
+        <v>168</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>168</v>
+        <v>185</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>169</v>
+        <v>186</v>
       </c>
       <c r="E59" s="12">
-        <v>45873</v>
+        <v>45819</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>81</v>
+        <v>181</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="I59" s="1" t="s">
         <v>80</v>
@@ -5149,16 +5154,16 @@
         <v>81</v>
       </c>
       <c r="N59" s="1">
-        <v>-817632</v>
+        <v>-2395</v>
       </c>
       <c r="O59" s="1">
-        <v>-701830</v>
+        <v>-2013</v>
       </c>
       <c r="P59" s="1">
         <v>0</v>
       </c>
       <c r="Q59" s="1">
-        <v>-133348</v>
+        <v>-382</v>
       </c>
       <c r="R59" s="1">
         <v>0</v>
@@ -5167,7 +5172,7 @@
         <v>0</v>
       </c>
       <c r="T59" s="1">
-        <v>17546</v>
+        <v>0</v>
       </c>
       <c r="U59" s="1">
         <v>0</v>
@@ -5213,25 +5218,25 @@
         <v>381</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>109</v>
+        <v>168</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>170</v>
+        <v>187</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>171</v>
+        <v>188</v>
       </c>
       <c r="E60" s="12">
-        <v>45873</v>
+        <v>45819</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>81</v>
+        <v>181</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>81</v>
+        <v>110</v>
       </c>
       <c r="I60" s="1" t="s">
         <v>80</v>
@@ -5249,16 +5254,16 @@
         <v>81</v>
       </c>
       <c r="N60" s="1">
-        <v>-3353617</v>
+        <v>-754</v>
       </c>
       <c r="O60" s="1">
-        <v>-2878641</v>
+        <v>-634</v>
       </c>
       <c r="P60" s="1">
         <v>0</v>
       </c>
       <c r="Q60" s="1">
-        <v>-546942</v>
+        <v>-120</v>
       </c>
       <c r="R60" s="1">
         <v>0</v>
@@ -5267,7 +5272,7 @@
         <v>0</v>
       </c>
       <c r="T60" s="1">
-        <v>71966</v>
+        <v>0</v>
       </c>
       <c r="U60" s="1">
         <v>0</v>
@@ -5313,25 +5318,25 @@
         <v>381</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>109</v>
+        <v>168</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>172</v>
+        <v>189</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>173</v>
+        <v>190</v>
       </c>
       <c r="E61" s="12">
-        <v>45873</v>
+        <v>45819</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>81</v>
+        <v>181</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>81</v>
+        <v>120</v>
       </c>
       <c r="I61" s="1" t="s">
         <v>80</v>
@@ -5349,16 +5354,16 @@
         <v>81</v>
       </c>
       <c r="N61" s="1">
-        <v>-13687887</v>
+        <v>-634</v>
       </c>
       <c r="O61" s="1">
-        <v>-11749260</v>
+        <v>-533</v>
       </c>
       <c r="P61" s="1">
         <v>0</v>
       </c>
       <c r="Q61" s="1">
-        <v>-2232359</v>
+        <v>-101</v>
       </c>
       <c r="R61" s="1">
         <v>0</v>
@@ -5367,7 +5372,7 @@
         <v>0</v>
       </c>
       <c r="T61" s="1">
-        <v>293732</v>
+        <v>0</v>
       </c>
       <c r="U61" s="1">
         <v>0</v>
@@ -5413,25 +5418,25 @@
         <v>381</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>109</v>
+        <v>168</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>174</v>
+        <v>191</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>175</v>
+        <v>192</v>
       </c>
       <c r="E62" s="12">
-        <v>45873</v>
+        <v>45820</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>81</v>
+        <v>131</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>81</v>
+        <v>193</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>81</v>
+        <v>142</v>
       </c>
       <c r="I62" s="1" t="s">
         <v>80</v>
@@ -5449,16 +5454,16 @@
         <v>81</v>
       </c>
       <c r="N62" s="1">
-        <v>-14589753</v>
+        <v>-289187</v>
       </c>
       <c r="O62" s="1">
-        <v>-12523393</v>
+        <v>-243014</v>
       </c>
       <c r="P62" s="1">
         <v>0</v>
       </c>
       <c r="Q62" s="1">
-        <v>-2379445</v>
+        <v>-46173</v>
       </c>
       <c r="R62" s="1">
         <v>0</v>
@@ -5467,7 +5472,7 @@
         <v>0</v>
       </c>
       <c r="T62" s="1">
-        <v>313085</v>
+        <v>0</v>
       </c>
       <c r="U62" s="1">
         <v>0</v>
@@ -5513,25 +5518,25 @@
         <v>381</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>109</v>
+        <v>168</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>176</v>
+        <v>194</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>177</v>
+        <v>195</v>
       </c>
       <c r="E63" s="12">
-        <v>45873</v>
+        <v>45820</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>81</v>
+        <v>131</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>81</v>
+        <v>193</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>81</v>
+        <v>153</v>
       </c>
       <c r="I63" s="1" t="s">
         <v>80</v>
@@ -5549,16 +5554,16 @@
         <v>81</v>
       </c>
       <c r="N63" s="1">
-        <v>-16674003</v>
+        <v>-909</v>
       </c>
       <c r="O63" s="1">
-        <v>-14312449</v>
+        <v>-764</v>
       </c>
       <c r="P63" s="1">
         <v>0</v>
       </c>
       <c r="Q63" s="1">
-        <v>-2719365</v>
+        <v>-145</v>
       </c>
       <c r="R63" s="1">
         <v>0</v>
@@ -5567,7 +5572,7 @@
         <v>0</v>
       </c>
       <c r="T63" s="1">
-        <v>357811</v>
+        <v>0</v>
       </c>
       <c r="U63" s="1">
         <v>0</v>
@@ -5613,25 +5618,25 @@
         <v>381</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>109</v>
+        <v>168</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>178</v>
+        <v>196</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>179</v>
+        <v>197</v>
       </c>
       <c r="E64" s="12">
-        <v>45873</v>
+        <v>45821</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>81</v>
+        <v>126</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>81</v>
+        <v>198</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>81</v>
+        <v>156</v>
       </c>
       <c r="I64" s="1" t="s">
         <v>80</v>
@@ -5649,16 +5654,16 @@
         <v>81</v>
       </c>
       <c r="N64" s="1">
-        <v>-19800379</v>
+        <v>-1597</v>
       </c>
       <c r="O64" s="1">
-        <v>-16996034</v>
+        <v>-1342</v>
       </c>
       <c r="P64" s="1">
         <v>0</v>
       </c>
       <c r="Q64" s="1">
-        <v>-3229246</v>
+        <v>-255</v>
       </c>
       <c r="R64" s="1">
         <v>0</v>
@@ -5667,7 +5672,7 @@
         <v>0</v>
       </c>
       <c r="T64" s="1">
-        <v>424901</v>
+        <v>0</v>
       </c>
       <c r="U64" s="1">
         <v>0</v>
@@ -5713,25 +5718,25 @@
         <v>381</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>109</v>
+        <v>168</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="E65" s="12">
-        <v>45873</v>
+        <v>45821</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>81</v>
+        <v>126</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>81</v>
+        <v>198</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>81</v>
+        <v>167</v>
       </c>
       <c r="I65" s="1" t="s">
         <v>80</v>
@@ -5749,16 +5754,16 @@
         <v>81</v>
       </c>
       <c r="N65" s="1">
-        <v>-21786554</v>
+        <v>-368</v>
       </c>
       <c r="O65" s="1">
-        <v>-18700905</v>
+        <v>-309</v>
       </c>
       <c r="P65" s="1">
         <v>0</v>
       </c>
       <c r="Q65" s="1">
-        <v>-3553172</v>
+        <v>-59</v>
       </c>
       <c r="R65" s="1">
         <v>0</v>
@@ -5767,7 +5772,7 @@
         <v>0</v>
       </c>
       <c r="T65" s="1">
-        <v>467523</v>
+        <v>0</v>
       </c>
       <c r="U65" s="1">
         <v>0</v>
@@ -5809,56 +5814,32 @@
       <c r="AN65" s="1"/>
     </row>
     <row r="66" spans="1:40" x14ac:dyDescent="0.3">
-      <c r="A66" s="1">
-        <v>381</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="E66" s="12">
-        <v>45873</v>
-      </c>
-      <c r="F66" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="G66" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="H66" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="I66" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="J66" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="K66" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="L66" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="M66" s="1" t="s">
-        <v>81</v>
-      </c>
+      <c r="A66" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B66" s="1"/>
+      <c r="C66" s="1"/>
+      <c r="D66" s="1"/>
+      <c r="E66" s="1"/>
+      <c r="F66" s="1"/>
+      <c r="G66" s="1"/>
+      <c r="H66" s="1"/>
+      <c r="I66" s="1"/>
+      <c r="J66" s="1"/>
+      <c r="K66" s="1"/>
+      <c r="L66" s="1"/>
+      <c r="M66" s="1"/>
       <c r="N66" s="1">
-        <v>-47451687</v>
+        <v>1188745461</v>
       </c>
       <c r="O66" s="1">
-        <v>-40731062</v>
+        <v>1000803412</v>
       </c>
       <c r="P66" s="1">
         <v>0</v>
       </c>
       <c r="Q66" s="1">
-        <v>-7738902</v>
+        <v>187942049</v>
       </c>
       <c r="R66" s="1">
         <v>0</v>
@@ -5867,7 +5848,7 @@
         <v>0</v>
       </c>
       <c r="T66" s="1">
-        <v>1018277</v>
+        <v>0</v>
       </c>
       <c r="U66" s="1">
         <v>0</v>
@@ -5886,795 +5867,19 @@
       </c>
       <c r="Z66" s="1"/>
       <c r="AA66" s="1"/>
-      <c r="AB66" s="1">
-        <v>0</v>
-      </c>
+      <c r="AB66" s="1"/>
       <c r="AC66" s="1"/>
-      <c r="AD66" s="1">
-        <v>0</v>
-      </c>
+      <c r="AD66" s="1"/>
       <c r="AE66" s="1"/>
-      <c r="AF66" s="1" t="s">
-        <v>83</v>
-      </c>
+      <c r="AF66" s="1"/>
       <c r="AG66" s="1"/>
-      <c r="AH66" s="1" t="s">
-        <v>84</v>
-      </c>
+      <c r="AH66" s="1"/>
       <c r="AI66" s="1"/>
       <c r="AJ66" s="1"/>
       <c r="AK66" s="1"/>
       <c r="AL66" s="1"/>
       <c r="AM66" s="1"/>
       <c r="AN66" s="1"/>
-    </row>
-    <row r="67" spans="1:40" x14ac:dyDescent="0.3">
-      <c r="A67" s="1">
-        <v>381</v>
-      </c>
-      <c r="B67" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="E67" s="12">
-        <v>45873</v>
-      </c>
-      <c r="F67" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="G67" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="H67" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="I67" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="J67" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="K67" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="L67" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="M67" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="N67" s="1">
-        <v>-54866013</v>
-      </c>
-      <c r="O67" s="1">
-        <v>-47095290</v>
-      </c>
-      <c r="P67" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q67" s="1">
-        <v>-8948105</v>
-      </c>
-      <c r="R67" s="1">
-        <v>0</v>
-      </c>
-      <c r="S67" s="1">
-        <v>0</v>
-      </c>
-      <c r="T67" s="1">
-        <v>1177382</v>
-      </c>
-      <c r="U67" s="1">
-        <v>0</v>
-      </c>
-      <c r="V67" s="1">
-        <v>0</v>
-      </c>
-      <c r="W67" s="1">
-        <v>0</v>
-      </c>
-      <c r="X67" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y67" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z67" s="1"/>
-      <c r="AA67" s="1"/>
-      <c r="AB67" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC67" s="1"/>
-      <c r="AD67" s="1">
-        <v>0</v>
-      </c>
-      <c r="AE67" s="1"/>
-      <c r="AF67" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="AG67" s="1"/>
-      <c r="AH67" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="AI67" s="1"/>
-      <c r="AJ67" s="1"/>
-      <c r="AK67" s="1"/>
-      <c r="AL67" s="1"/>
-      <c r="AM67" s="1"/>
-      <c r="AN67" s="1"/>
-    </row>
-    <row r="68" spans="1:40" x14ac:dyDescent="0.3">
-      <c r="A68" s="1">
-        <v>381</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C68" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="D68" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="E68" s="12">
-        <v>45873</v>
-      </c>
-      <c r="F68" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="G68" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="H68" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="I68" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="J68" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="K68" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="L68" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="M68" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="N68" s="1">
-        <v>-65740358</v>
-      </c>
-      <c r="O68" s="1">
-        <v>-56429492</v>
-      </c>
-      <c r="P68" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q68" s="1">
-        <v>-10721603</v>
-      </c>
-      <c r="R68" s="1">
-        <v>0</v>
-      </c>
-      <c r="S68" s="1">
-        <v>0</v>
-      </c>
-      <c r="T68" s="1">
-        <v>1410737</v>
-      </c>
-      <c r="U68" s="1">
-        <v>0</v>
-      </c>
-      <c r="V68" s="1">
-        <v>0</v>
-      </c>
-      <c r="W68" s="1">
-        <v>0</v>
-      </c>
-      <c r="X68" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y68" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z68" s="1"/>
-      <c r="AA68" s="1"/>
-      <c r="AB68" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC68" s="1"/>
-      <c r="AD68" s="1">
-        <v>0</v>
-      </c>
-      <c r="AE68" s="1"/>
-      <c r="AF68" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="AG68" s="1"/>
-      <c r="AH68" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="AI68" s="1"/>
-      <c r="AJ68" s="1"/>
-      <c r="AK68" s="1"/>
-      <c r="AL68" s="1"/>
-      <c r="AM68" s="1"/>
-      <c r="AN68" s="1"/>
-    </row>
-    <row r="69" spans="1:40" x14ac:dyDescent="0.3">
-      <c r="A69" s="1">
-        <v>381</v>
-      </c>
-      <c r="B69" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C69" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="D69" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="E69" s="12">
-        <v>45802</v>
-      </c>
-      <c r="F69" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="G69" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="H69" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="I69" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="J69" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="K69" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="L69" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="M69" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="N69" s="1">
-        <v>-2</v>
-      </c>
-      <c r="O69" s="1">
-        <v>-2</v>
-      </c>
-      <c r="P69" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q69" s="1">
-        <v>0</v>
-      </c>
-      <c r="R69" s="1">
-        <v>0</v>
-      </c>
-      <c r="S69" s="1">
-        <v>0</v>
-      </c>
-      <c r="T69" s="1">
-        <v>0</v>
-      </c>
-      <c r="U69" s="1">
-        <v>0</v>
-      </c>
-      <c r="V69" s="1">
-        <v>0</v>
-      </c>
-      <c r="W69" s="1">
-        <v>0</v>
-      </c>
-      <c r="X69" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y69" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z69" s="1"/>
-      <c r="AA69" s="1"/>
-      <c r="AB69" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC69" s="1"/>
-      <c r="AD69" s="1">
-        <v>0</v>
-      </c>
-      <c r="AE69" s="1"/>
-      <c r="AF69" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="AG69" s="1"/>
-      <c r="AH69" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="AI69" s="1"/>
-      <c r="AJ69" s="1"/>
-      <c r="AK69" s="1"/>
-      <c r="AL69" s="1"/>
-      <c r="AM69" s="1"/>
-      <c r="AN69" s="1"/>
-    </row>
-    <row r="70" spans="1:40" x14ac:dyDescent="0.3">
-      <c r="A70" s="1">
-        <v>381</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C70" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="D70" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="E70" s="12">
-        <v>45802</v>
-      </c>
-      <c r="F70" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="G70" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="H70" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="I70" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="J70" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="K70" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="L70" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="M70" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="N70" s="1">
-        <v>-143069</v>
-      </c>
-      <c r="O70" s="1">
-        <v>-120226</v>
-      </c>
-      <c r="P70" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q70" s="1">
-        <v>-22843</v>
-      </c>
-      <c r="R70" s="1">
-        <v>0</v>
-      </c>
-      <c r="S70" s="1">
-        <v>0</v>
-      </c>
-      <c r="T70" s="1">
-        <v>0</v>
-      </c>
-      <c r="U70" s="1">
-        <v>0</v>
-      </c>
-      <c r="V70" s="1">
-        <v>0</v>
-      </c>
-      <c r="W70" s="1">
-        <v>0</v>
-      </c>
-      <c r="X70" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y70" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z70" s="1"/>
-      <c r="AA70" s="1"/>
-      <c r="AB70" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC70" s="1"/>
-      <c r="AD70" s="1">
-        <v>0</v>
-      </c>
-      <c r="AE70" s="1"/>
-      <c r="AF70" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="AG70" s="1"/>
-      <c r="AH70" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="AI70" s="1"/>
-      <c r="AJ70" s="1"/>
-      <c r="AK70" s="1"/>
-      <c r="AL70" s="1"/>
-      <c r="AM70" s="1"/>
-      <c r="AN70" s="1"/>
-    </row>
-    <row r="71" spans="1:40" x14ac:dyDescent="0.3">
-      <c r="A71" s="1">
-        <v>381</v>
-      </c>
-      <c r="B71" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C71" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="D71" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="E71" s="12">
-        <v>45802</v>
-      </c>
-      <c r="F71" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="G71" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="H71" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="I71" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="J71" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="K71" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="L71" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="M71" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="N71" s="1">
-        <v>-9553281</v>
-      </c>
-      <c r="O71" s="1">
-        <v>-8027967</v>
-      </c>
-      <c r="P71" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q71" s="1">
-        <v>-1525314</v>
-      </c>
-      <c r="R71" s="1">
-        <v>0</v>
-      </c>
-      <c r="S71" s="1">
-        <v>0</v>
-      </c>
-      <c r="T71" s="1">
-        <v>0</v>
-      </c>
-      <c r="U71" s="1">
-        <v>0</v>
-      </c>
-      <c r="V71" s="1">
-        <v>0</v>
-      </c>
-      <c r="W71" s="1">
-        <v>0</v>
-      </c>
-      <c r="X71" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y71" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z71" s="1"/>
-      <c r="AA71" s="1"/>
-      <c r="AB71" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC71" s="1"/>
-      <c r="AD71" s="1">
-        <v>0</v>
-      </c>
-      <c r="AE71" s="1"/>
-      <c r="AF71" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="AG71" s="1"/>
-      <c r="AH71" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="AI71" s="1"/>
-      <c r="AJ71" s="1"/>
-      <c r="AK71" s="1"/>
-      <c r="AL71" s="1"/>
-      <c r="AM71" s="1"/>
-      <c r="AN71" s="1"/>
-    </row>
-    <row r="72" spans="1:40" x14ac:dyDescent="0.3">
-      <c r="A72" s="1">
-        <v>381</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C72" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="D72" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="E72" s="12">
-        <v>45803</v>
-      </c>
-      <c r="F72" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="G72" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="H72" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="I72" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="J72" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="K72" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="L72" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="M72" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="N72" s="1">
-        <v>-97382</v>
-      </c>
-      <c r="O72" s="1">
-        <v>-81834</v>
-      </c>
-      <c r="P72" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q72" s="1">
-        <v>-15548</v>
-      </c>
-      <c r="R72" s="1">
-        <v>0</v>
-      </c>
-      <c r="S72" s="1">
-        <v>0</v>
-      </c>
-      <c r="T72" s="1">
-        <v>0</v>
-      </c>
-      <c r="U72" s="1">
-        <v>0</v>
-      </c>
-      <c r="V72" s="1">
-        <v>0</v>
-      </c>
-      <c r="W72" s="1">
-        <v>0</v>
-      </c>
-      <c r="X72" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y72" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z72" s="1"/>
-      <c r="AA72" s="1"/>
-      <c r="AB72" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC72" s="1"/>
-      <c r="AD72" s="1">
-        <v>0</v>
-      </c>
-      <c r="AE72" s="1"/>
-      <c r="AF72" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="AG72" s="1"/>
-      <c r="AH72" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="AI72" s="1"/>
-      <c r="AJ72" s="1"/>
-      <c r="AK72" s="1"/>
-      <c r="AL72" s="1"/>
-      <c r="AM72" s="1"/>
-      <c r="AN72" s="1"/>
-    </row>
-    <row r="73" spans="1:40" x14ac:dyDescent="0.3">
-      <c r="A73" s="1">
-        <v>381</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C73" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="D73" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="E73" s="12">
-        <v>45803</v>
-      </c>
-      <c r="F73" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="G73" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="H73" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="I73" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="J73" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="K73" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="L73" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="M73" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="N73" s="1">
-        <v>-649</v>
-      </c>
-      <c r="O73" s="1">
-        <v>-545</v>
-      </c>
-      <c r="P73" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q73" s="1">
-        <v>-104</v>
-      </c>
-      <c r="R73" s="1">
-        <v>0</v>
-      </c>
-      <c r="S73" s="1">
-        <v>0</v>
-      </c>
-      <c r="T73" s="1">
-        <v>0</v>
-      </c>
-      <c r="U73" s="1">
-        <v>0</v>
-      </c>
-      <c r="V73" s="1">
-        <v>0</v>
-      </c>
-      <c r="W73" s="1">
-        <v>0</v>
-      </c>
-      <c r="X73" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y73" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z73" s="1"/>
-      <c r="AA73" s="1"/>
-      <c r="AB73" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC73" s="1"/>
-      <c r="AD73" s="1">
-        <v>0</v>
-      </c>
-      <c r="AE73" s="1"/>
-      <c r="AF73" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="AG73" s="1"/>
-      <c r="AH73" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="AI73" s="1"/>
-      <c r="AJ73" s="1"/>
-      <c r="AK73" s="1"/>
-      <c r="AL73" s="1"/>
-      <c r="AM73" s="1"/>
-      <c r="AN73" s="1"/>
-    </row>
-    <row r="74" spans="1:40" x14ac:dyDescent="0.3">
-      <c r="A74" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="B74" s="1"/>
-      <c r="C74" s="1"/>
-      <c r="D74" s="1"/>
-      <c r="E74" s="1"/>
-      <c r="F74" s="1"/>
-      <c r="G74" s="1"/>
-      <c r="H74" s="1"/>
-      <c r="I74" s="1"/>
-      <c r="J74" s="1"/>
-      <c r="K74" s="1"/>
-      <c r="L74" s="1"/>
-      <c r="M74" s="1"/>
-      <c r="N74" s="1">
-        <v>1047007047</v>
-      </c>
-      <c r="O74" s="1">
-        <v>826991292</v>
-      </c>
-      <c r="P74" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q74" s="1">
-        <v>214445249</v>
-      </c>
-      <c r="R74" s="1">
-        <v>0</v>
-      </c>
-      <c r="S74" s="1">
-        <v>0</v>
-      </c>
-      <c r="T74" s="1">
-        <v>5570506</v>
-      </c>
-      <c r="U74" s="1">
-        <v>0</v>
-      </c>
-      <c r="V74" s="1">
-        <v>0</v>
-      </c>
-      <c r="W74" s="1">
-        <v>0</v>
-      </c>
-      <c r="X74" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y74" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z74" s="1"/>
-      <c r="AA74" s="1"/>
-      <c r="AB74" s="1"/>
-      <c r="AC74" s="1"/>
-      <c r="AD74" s="1"/>
-      <c r="AE74" s="1"/>
-      <c r="AF74" s="1"/>
-      <c r="AG74" s="1"/>
-      <c r="AH74" s="1"/>
-      <c r="AI74" s="1"/>
-      <c r="AJ74" s="1"/>
-      <c r="AK74" s="1"/>
-      <c r="AL74" s="1"/>
-      <c r="AM74" s="1"/>
-      <c r="AN74" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -6692,291 +5897,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010050AE9A0F24DEC94E918D544AFEE50C64" ma:contentTypeVersion="17" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="ad041989b7b6f045e3e28b9562348916">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="04da54ee-f080-44b9-94d6-1e4751f8e229" xmlns:ns3="1b1d4eed-8783-4e89-ad60-9f4bc6bec550" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5bade24fc5071da01a1452a5e025067a" ns2:_="" ns3:_="">
-    <xsd:import namespace="04da54ee-f080-44b9-94d6-1e4751f8e229"/>
-    <xsd:import namespace="1b1d4eed-8783-4e89-ad60-9f4bc6bec550"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="04da54ee-f080-44b9-94d6-1e4751f8e229" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="12" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceKeyPoints" ma:index="13" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="15" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="b7f554e9-a963-4179-93d8-b97c19740184" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="18" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="19" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="20" nillable="true" ma:displayName="MediaServiceDateTaken" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="21" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="22" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="23" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="24" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="1b1d4eed-8783-4e89-ad60-9f4bc6bec550" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="10" nillable="true" ma:displayName="Compartido con" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="11" nillable="true" ma:displayName="Detalles de uso compartido" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="TaxCatchAll" ma:index="16" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{aa2d1a3a-e7df-457d-bf05-60da16be1a98}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="1b1d4eed-8783-4e89-ad60-9f4bc6bec550">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="04da54ee-f080-44b9-94d6-1e4751f8e229">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="1b1d4eed-8783-4e89-ad60-9f4bc6bec550" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5055192E-A4C7-4044-944F-1186E4ABE945}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24FD46EA-20D0-4E8B-A70D-324DBEF76533}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D80F067B-2FC5-4EF7-963B-394BA9DE5133}"/>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{89db4e91-bad5-4fd0-9ca4-c06485916e3a}" enabled="1" method="Standard" siteId="{f66fae02-5d36-495b-bfe0-78a6ff9f8e6e}" removed="0"/>
-</clbl:labelList>
 </file>
</xml_diff>